<commit_message>
Lab-6 & logical,relational and conditional operator done successfully
</commit_message>
<xml_diff>
--- a/Conditional Formatting.xlsx
+++ b/Conditional Formatting.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\N327_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{236776A5-AD68-4D0B-9264-1B15E13F2124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D736258F-2614-40A3-BCF1-3AC0F80BEB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{AD6C997B-D305-4C51-8C4D-0A33C7475563}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{AD6C997B-D305-4C51-8C4D-0A33C7475563}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="LOGICAL OPERATORS" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="88">
   <si>
     <t>Name</t>
   </si>
@@ -151,13 +152,270 @@
   </si>
   <si>
     <t>Vivaan</t>
+  </si>
+  <si>
+    <t>Meanings</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
+  <si>
+    <t>Equals to</t>
+  </si>
+  <si>
+    <t>&lt;</t>
+  </si>
+  <si>
+    <t>Less Than</t>
+  </si>
+  <si>
+    <t>Less Than Equals to</t>
+  </si>
+  <si>
+    <t>&lt;=</t>
+  </si>
+  <si>
+    <t>&gt;=</t>
+  </si>
+  <si>
+    <t>Greater than equals to</t>
+  </si>
+  <si>
+    <t>&gt;</t>
+  </si>
+  <si>
+    <t>Greater than</t>
+  </si>
+  <si>
+    <t>&lt;&gt;</t>
+  </si>
+  <si>
+    <t>Logical Operators</t>
+  </si>
+  <si>
+    <t>G5=10</t>
+  </si>
+  <si>
+    <t>G5&lt;15</t>
+  </si>
+  <si>
+    <t>G5&lt;=15</t>
+  </si>
+  <si>
+    <t>G5&gt;=15</t>
+  </si>
+  <si>
+    <t>G5&lt;&gt;15</t>
+  </si>
+  <si>
+    <t>G5&gt;19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not </t>
+  </si>
+  <si>
+    <t>Relational Operators</t>
+  </si>
+  <si>
+    <t>AND</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>NOT</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>all condition is True</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> then it returns </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>True</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> otherwise </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>False</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>any of the condition is True</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> it returns </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>True</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> otherwise </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>False</t>
+    </r>
+  </si>
+  <si>
+    <t>It just reverse the results</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Instock</t>
+  </si>
+  <si>
+    <t>Sold</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Banana</t>
+  </si>
+  <si>
+    <t>Oranges</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>IF Formula with AND operator</t>
+  </si>
+  <si>
+    <t>IF formula with OR operator</t>
+  </si>
+  <si>
+    <t>sub2</t>
+  </si>
+  <si>
+    <t>Akash</t>
+  </si>
+  <si>
+    <t>Heena</t>
+  </si>
+  <si>
+    <t>sub1</t>
+  </si>
+  <si>
+    <t>Not Operator</t>
+  </si>
+  <si>
+    <t>Num1</t>
+  </si>
+  <si>
+    <t>Num2</t>
+  </si>
+  <si>
+    <t>div</t>
+  </si>
+  <si>
+    <t>div with iferror()</t>
+  </si>
+  <si>
+    <t>add with iferror()</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>Multiply with iferror()</t>
+  </si>
+  <si>
+    <t>iferror with subtraction</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +439,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -196,10 +461,36 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -208,23 +499,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="5">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -245,56 +560,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -881,18 +1146,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H8">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
-      <formula>"Pass"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B2:E8">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
-      <formula>40</formula>
-    </cfRule>
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -904,6 +1158,17 @@
           <x14:id>{5C391DFE-A61F-4369-8EE6-3537ABFAA461}</x14:id>
         </ext>
       </extLst>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>40</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H8">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -929,14 +1194,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44ABC048-1EB4-4FB2-AC74-6608647083D7}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.7265625" customWidth="1"/>
     <col min="2" max="2" width="18.453125" customWidth="1"/>
+    <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -944,7 +1210,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -952,7 +1218,7 @@
         <v>46003</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -960,7 +1226,7 @@
         <v>46223</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -968,15 +1234,19 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="3">
         <v>46338</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F5" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -984,7 +1254,7 @@
         <v>46336</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -992,7 +1262,7 @@
         <v>46216</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1000,7 +1270,7 @@
         <v>45853</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1008,7 +1278,7 @@
         <v>45854</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1016,7 +1286,7 @@
         <v>45855</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1024,7 +1294,7 @@
         <v>45856</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1032,7 +1302,7 @@
         <v>45857</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -1040,7 +1310,7 @@
         <v>45858</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -1048,7 +1318,7 @@
         <v>45859</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1056,7 +1326,7 @@
         <v>45860</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1110,6 +1380,526 @@
       </c>
       <c r="B22" s="3">
         <v>46355</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A22">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$B$2:$B$22&gt;TODAY()</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>$B$2:$B$22&lt;=TODAY()</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65577E96-2764-4630-A96C-E50102812DEB}">
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.81640625" customWidth="1"/>
+    <col min="2" max="2" width="11.6328125" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" customWidth="1"/>
+    <col min="4" max="4" width="13.7265625" customWidth="1"/>
+    <col min="5" max="5" width="14.1796875" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
+    <col min="7" max="7" width="22.6328125" customWidth="1"/>
+    <col min="8" max="8" width="26.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="23" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="4" t="b">
+        <f>G5=10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="4" t="b">
+        <f>G5&lt;15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="4" t="b">
+        <f>G5&lt;=15</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="4" t="b">
+        <f>G5&gt;=15</f>
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="4" t="b">
+        <f>G5&gt;19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="4" t="b">
+        <f>G5&lt;&gt;15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="4">
+        <v>30</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11" t="b">
+        <f>AND(C11="Banana",D11&gt;E11)</f>
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <f>IF(AND(C11="Banana",D11&gt;E11),"Able to Sold","Out of Stock")</f>
+        <v>Able to Sold</v>
+      </c>
+      <c r="H11" t="str">
+        <f>IF(OR(C11="Banana",D11&lt;E11),"Able to Sold","Out of Stock")</f>
+        <v>Able to Sold</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="4">
+        <v>40</v>
+      </c>
+      <c r="E12">
+        <v>40</v>
+      </c>
+      <c r="F12" t="b">
+        <f>AND(C12="Oranges",D12&gt;E12)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" t="str">
+        <f>IF(AND(C12="Oranges",D12&gt;E12),"Able to Sold","Out of Stock")</f>
+        <v>Out of Stock</v>
+      </c>
+      <c r="H12" t="str">
+        <f>IF(OR(C12="Mango",D12&lt;E12),"out of stock","Product is not available")</f>
+        <v>Product is not available</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="4">
+        <v>40</v>
+      </c>
+      <c r="E13">
+        <v>10</v>
+      </c>
+      <c r="F13" t="b">
+        <f>AND(C13="Banana",D13&gt;E13)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" t="str">
+        <f>IF(AND(C13="Apple",D13&gt;E13),"Able to Sold","Out of Stock")</f>
+        <v>Able to Sold</v>
+      </c>
+      <c r="H13" t="str">
+        <f>IF(OR(C13="Apple",D13&gt;E13),"Able to Sold","Out of Stock")</f>
+        <v>Able to Sold</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="10">
+        <v>45</v>
+      </c>
+      <c r="C21" s="10">
+        <v>50</v>
+      </c>
+      <c r="D21" s="10" t="str">
+        <f>IF(AND(B21&gt;40,C21&gt;40),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="E21" s="4" t="str">
+        <f>IF(NOT(AND(B21&gt;40,C21&gt;40)),"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="10">
+        <v>34</v>
+      </c>
+      <c r="C22" s="10">
+        <v>41</v>
+      </c>
+      <c r="D22" s="10" t="str">
+        <f t="shared" ref="D22:D24" si="0">IF(AND(B22&gt;40,C22&gt;40),"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="E22" s="4" t="str">
+        <f t="shared" ref="E22:E24" si="1">IF(NOT(AND(B22&gt;40,C22&gt;40)),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" s="10">
+        <v>56</v>
+      </c>
+      <c r="C23" s="10">
+        <v>58</v>
+      </c>
+      <c r="D23" s="10" t="str">
+        <f t="shared" si="0"/>
+        <v>Pass</v>
+      </c>
+      <c r="E23" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" s="10">
+        <v>41</v>
+      </c>
+      <c r="C24" s="10">
+        <v>56</v>
+      </c>
+      <c r="D24" s="10" t="str">
+        <f t="shared" si="0"/>
+        <v>Pass</v>
+      </c>
+      <c r="E24" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>10</v>
+      </c>
+      <c r="B27" s="11">
+        <v>2</v>
+      </c>
+      <c r="C27">
+        <f>A27/B27</f>
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <f>IFERROR(A27/B27,"Not divisible by zero")</f>
+        <v>5</v>
+      </c>
+      <c r="E27">
+        <f>IFERROR(A27*B27,"unable to multiply")</f>
+        <v>20</v>
+      </c>
+      <c r="F27">
+        <f>IFERROR(A27+B27,"unable to add")</f>
+        <v>12</v>
+      </c>
+      <c r="G27">
+        <f>IFERROR(A27-B27,"unable to perform subtraction")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>19</v>
+      </c>
+      <c r="B28" s="11">
+        <v>8</v>
+      </c>
+      <c r="C28">
+        <f t="shared" ref="C28:C30" si="2">A28/B28</f>
+        <v>2.375</v>
+      </c>
+      <c r="D28">
+        <f t="shared" ref="D28:D30" si="3">IFERROR(A28/B28,"Not divisible by zero")</f>
+        <v>2.375</v>
+      </c>
+      <c r="E28">
+        <f t="shared" ref="E28:E31" si="4">IFERROR(A28*B28,"unable to multiply")</f>
+        <v>152</v>
+      </c>
+      <c r="F28">
+        <f t="shared" ref="F28:F31" si="5">IFERROR(A28+B28,"unable to add")</f>
+        <v>27</v>
+      </c>
+      <c r="G28">
+        <f t="shared" ref="G28:G31" si="6">IFERROR(A28-B28,"unable to perform subtraction")</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>0</v>
+      </c>
+      <c r="B29" s="11">
+        <v>23</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="5"/>
+        <v>23</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="6"/>
+        <v>-23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>144</v>
+      </c>
+      <c r="B30" s="11">
+        <v>0</v>
+      </c>
+      <c r="C30" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D30" t="str">
+        <f t="shared" si="3"/>
+        <v>Not divisible by zero</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="6"/>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>85</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="4"/>
+        <v>unable to multiply</v>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="5"/>
+        <v>unable to add</v>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="6"/>
+        <v>unable to perform subtraction</v>
       </c>
     </row>
   </sheetData>

</xml_diff>